<commit_message>
Add and verify dazai and Resolushh partner UTM links
</commit_message>
<xml_diff>
--- a/docs/utm.xlsx
+++ b/docs/utm.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utm" sheetId="1" r:id="R7c416b836a1246ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utm" sheetId="1" r:id="Rcc47cd0b10e74828"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -83,7 +83,7 @@
   <x:dxfs count="1">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CC"/>
         </x:patternFill>
       </x:fill>
@@ -783,7 +783,9 @@
       <x:c r="C11" s="6" t="str">
         <x:v>Партнёрская публикация</x:v>
       </x:c>
-      <x:c r="D11" s="7" t="str"/>
+      <x:c r="D11" s="7" t="str">
+        <x:v>dazai</x:v>
+      </x:c>
       <x:c r="E11" s="7" t="str">
         <x:v>affiliate</x:v>
       </x:c>
@@ -801,15 +803,16 @@
       </x:c>
       <x:c r="J11" s="6" t="str">
         <x:f>IF(D11="","",$R$2&amp;"/"&amp;I11&amp;"?utm_source="&amp;D11&amp;"&amp;utm_medium="&amp;E11&amp;"&amp;utm_campaign="&amp;F11&amp;"&amp;utm_content="&amp;G11&amp;IF(H11="","","&amp;utm_term="&amp;H11)&amp;IF(P11="","","#"&amp;P11))</x:f>
+        <x:v>https://tz-11-turklub-tropa-phi.vercel.app/index.html?utm_source=dazai&amp;utm_medium=affiliate&amp;utm_campaign=winter_trips_2026&amp;utm_content=stories_01&amp;utm_term=winter_hiking</x:v>
       </x:c>
       <x:c r="K11" s="6"/>
       <x:c r="L11" s="6"/>
       <x:c r="M11" s="6"/>
       <x:c r="N11" s="6" t="str">
-        <x:v>Отложено пользователем</x:v>
+        <x:v>Переход проверен 30.10.2026; учебная ссылка</x:v>
       </x:c>
       <x:c r="O11" s="6" t="str">
-        <x:v>Нужен ник первого одногруппника</x:v>
+        <x:v>Главная страница знакомит с клубом и помогает выбрать поход</x:v>
       </x:c>
       <x:c r="P11" s="6" t="str"/>
       <x:c r="Q11" s="1"/>
@@ -825,7 +828,9 @@
       <x:c r="C12" s="6" t="str">
         <x:v>Партнёрская публикация</x:v>
       </x:c>
-      <x:c r="D12" s="7" t="str"/>
+      <x:c r="D12" s="7" t="str">
+        <x:v>resolushh</x:v>
+      </x:c>
       <x:c r="E12" s="7" t="str">
         <x:v>affiliate</x:v>
       </x:c>
@@ -843,15 +848,16 @@
       </x:c>
       <x:c r="J12" s="6" t="str">
         <x:f>IF(D12="","",$R$2&amp;"/"&amp;I12&amp;"?utm_source="&amp;D12&amp;"&amp;utm_medium="&amp;E12&amp;"&amp;utm_campaign="&amp;F12&amp;"&amp;utm_content="&amp;G12&amp;IF(H12="","","&amp;utm_term="&amp;H12)&amp;IF(P12="","","#"&amp;P12))</x:f>
+        <x:v>https://tz-11-turklub-tropa-phi.vercel.app/gear.html?utm_source=resolushh&amp;utm_medium=affiliate&amp;utm_campaign=winter_trips_2026&amp;utm_content=post_01&amp;utm_term=winter_hiking</x:v>
       </x:c>
       <x:c r="K12" s="6"/>
       <x:c r="L12" s="6"/>
       <x:c r="M12" s="6"/>
       <x:c r="N12" s="6" t="str">
-        <x:v>Отложено пользователем</x:v>
+        <x:v>Переход проверен 30.10.2026; учебная ссылка</x:v>
       </x:c>
       <x:c r="O12" s="6" t="str">
-        <x:v>Нужен ник второго одногруппника</x:v>
+        <x:v>Чек-лист и калькулятор аренды для подготовки к походу</x:v>
       </x:c>
       <x:c r="P12" s="6" t="str"/>
       <x:c r="Q12" s="1"/>

</xml_diff>

<commit_message>
Finalize course documentation with current evidence and limits
</commit_message>
<xml_diff>
--- a/docs/utm.xlsx
+++ b/docs/utm.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utm" sheetId="1" r:id="Rcc47cd0b10e74828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="utm" sheetId="1" r:id="Rf2fd9d5621e340d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -440,10 +440,14 @@
         <x:v>https://tz-11-turklub-tropa-phi.vercel.app/gear.html?utm_source=instagram&amp;utm_medium=social&amp;utm_campaign=winter_trips_2026&amp;utm_content=reel_tent_01&amp;utm_term=winter_hiking</x:v>
       </x:c>
       <x:c r="K3" s="6"/>
-      <x:c r="L3" s="6"/>
-      <x:c r="M3" s="6"/>
+      <x:c r="L3" s="6" t="str">
+        <x:v>https://www.instagram.com/reel/DfFy1SzKrMz/</x:v>
+      </x:c>
+      <x:c r="M3" s="6" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>Подготовлена, не опубликована</x:v>
+        <x:v>ManyChat Live; Direct и переход проверены; заявка СНАРЯГА подтверждена</x:v>
       </x:c>
       <x:c r="O3" s="6" t="str">
         <x:v>Чек-лист и калькулятор</x:v>
@@ -487,10 +491,14 @@
         <x:v>https://tz-11-turklub-tropa-phi.vercel.app/trips.html?utm_source=instagram&amp;utm_medium=social&amp;utm_campaign=beginners_dec_2026&amp;utm_content=reel_tent_01_easy&amp;utm_term=winter_hiking#easy</x:v>
       </x:c>
       <x:c r="K4" s="6"/>
-      <x:c r="L4" s="6"/>
-      <x:c r="M4" s="6"/>
+      <x:c r="L4" s="6" t="str">
+        <x:v>https://www.instagram.com/reel/DfFy1SzKrMz/</x:v>
+      </x:c>
+      <x:c r="M4" s="6" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
       <x:c r="N4" s="6" t="str">
-        <x:v>Подготовлена, не опубликована</x:v>
+        <x:v>ManyChat Live; Direct и переход проверены; заявка НОВИЧОК отдельно не проверена</x:v>
       </x:c>
       <x:c r="O4" s="6" t="str">
         <x:v>Три лёгких маршрута</x:v>

</xml_diff>